<commit_message>
xlsx download wowking good
</commit_message>
<xml_diff>
--- a/IO/sample/op_sample.xlsx
+++ b/IO/sample/op_sample.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
   <si>
     <t xml:space="preserve">S. NO. </t>
   </si>
@@ -153,9 +153,6 @@
   </si>
   <si>
     <t>LD#3 &amp; TSCR</t>
-  </si>
-  <si>
-    <t>RATE/HR</t>
   </si>
   <si>
     <t>NET LOSS:</t>
@@ -2680,38 +2677,22 @@
     </row>
     <row r="20" s="1" customFormat="1" spans="1:18">
       <c r="A20" s="10"/>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="11"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="12"/>
+      <c r="Q20" s="17" t="s">
         <v>42</v>
-      </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="12">
-        <v>2564.1</v>
-      </c>
-      <c r="E20" s="10"/>
-      <c r="F20" s="12">
-        <v>1602.56</v>
-      </c>
-      <c r="G20" s="10"/>
-      <c r="H20" s="12">
-        <v>1362.18</v>
-      </c>
-      <c r="J20" s="12">
-        <v>1442.31</v>
-      </c>
-      <c r="K20" s="10"/>
-      <c r="L20" s="12">
-        <v>1350</v>
-      </c>
-      <c r="M20" s="10"/>
-      <c r="N20" s="12">
-        <v>2628</v>
-      </c>
-      <c r="O20" s="10"/>
-      <c r="P20" s="12">
-        <v>4247</v>
-      </c>
-      <c r="Q20" s="17" t="s">
-        <v>43</v>
       </c>
       <c r="R20" s="18">
         <f>SUM(R2:R19)</f>

</xml_diff>